<commit_message>
Actualizacao dos graficos da pagina visao geral
</commit_message>
<xml_diff>
--- a/Lista_Nacala_Porto_Turmas.xlsx
+++ b/Lista_Nacala_Porto_Turmas.xlsx
@@ -1,20 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://muvamozorg.sharepoint.com/sites/mis.drive/Documentos Partilhados/PROJECTOS/Sistema de Monitoria/NEXUS/2026/Dash_Nexus/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="52" documentId="8_{F0ECD2CA-1AFC-4D72-92BC-085899DFC072}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{806549D5-C47C-415C-A3F4-07E5F9C9B417}"/>
+  <xr:revisionPtr revIDLastSave="53" documentId="8_{F0ECD2CA-1AFC-4D72-92BC-085899DFC072}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{72CCFE79-889A-4ACC-8210-E6E1F573723B}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{619861BA-25F5-43D2-A075-305249973C9B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$G$250</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -1469,16 +1472,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{156349CF-6280-4CD0-803A-013CF8C0A2F2}">
   <dimension ref="A1:G250"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="40.21875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.21875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="40.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.1796875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="28" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1501,7 +1504,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="12" t="s">
         <v>42</v>
       </c>
@@ -1524,7 +1527,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="12" t="s">
         <v>42</v>
       </c>
@@ -1547,7 +1550,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="12" t="s">
         <v>42</v>
       </c>
@@ -1570,7 +1573,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="12" t="s">
         <v>42</v>
       </c>
@@ -1593,7 +1596,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" s="12" t="s">
         <v>42</v>
       </c>
@@ -1616,7 +1619,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="7" t="s">
         <v>42</v>
       </c>
@@ -1639,7 +1642,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" s="7" t="s">
         <v>42</v>
       </c>
@@ -1662,7 +1665,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" s="7" t="s">
         <v>42</v>
       </c>
@@ -1685,7 +1688,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" s="7" t="s">
         <v>42</v>
       </c>
@@ -1708,7 +1711,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" s="7" t="s">
         <v>42</v>
       </c>
@@ -1731,7 +1734,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" s="7" t="s">
         <v>42</v>
       </c>
@@ -1754,7 +1757,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" s="7" t="s">
         <v>42</v>
       </c>
@@ -1777,7 +1780,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" s="7" t="s">
         <v>42</v>
       </c>
@@ -1800,7 +1803,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" s="7" t="s">
         <v>42</v>
       </c>
@@ -1823,7 +1826,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" s="7" t="s">
         <v>42</v>
       </c>
@@ -1846,7 +1849,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" s="7" t="s">
         <v>42</v>
       </c>
@@ -1869,7 +1872,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18" s="7" t="s">
         <v>42</v>
       </c>
@@ -1892,7 +1895,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" s="7" t="s">
         <v>42</v>
       </c>
@@ -1915,7 +1918,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A20" s="7" t="s">
         <v>42</v>
       </c>
@@ -1938,7 +1941,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" s="7" t="s">
         <v>42</v>
       </c>
@@ -1961,7 +1964,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A22" s="7" t="s">
         <v>42</v>
       </c>
@@ -1984,7 +1987,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A23" s="7" t="s">
         <v>42</v>
       </c>
@@ -2007,7 +2010,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24" s="7" t="s">
         <v>42</v>
       </c>
@@ -2030,7 +2033,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25" s="7" t="s">
         <v>42</v>
       </c>
@@ -2053,7 +2056,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A26" s="7" t="s">
         <v>42</v>
       </c>
@@ -2076,7 +2079,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27" s="7" t="s">
         <v>42</v>
       </c>
@@ -2099,7 +2102,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A28" s="7" t="s">
         <v>42</v>
       </c>
@@ -2122,7 +2125,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A29" s="7" t="s">
         <v>42</v>
       </c>
@@ -2145,7 +2148,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A30" s="7" t="s">
         <v>42</v>
       </c>
@@ -2168,7 +2171,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A31" s="7" t="s">
         <v>42</v>
       </c>
@@ -2191,7 +2194,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32" s="7" t="s">
         <v>42</v>
       </c>
@@ -2214,7 +2217,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A33" s="7" t="s">
         <v>42</v>
       </c>
@@ -2237,7 +2240,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A34" s="7" t="s">
         <v>42</v>
       </c>
@@ -2260,7 +2263,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A35" s="7" t="s">
         <v>42</v>
       </c>
@@ -2283,7 +2286,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A36" s="7" t="s">
         <v>42</v>
       </c>
@@ -2306,7 +2309,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A37" s="7" t="s">
         <v>42</v>
       </c>
@@ -2329,7 +2332,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A38" s="7" t="s">
         <v>42</v>
       </c>
@@ -2352,7 +2355,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A39" s="7" t="s">
         <v>42</v>
       </c>
@@ -2375,7 +2378,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A40" s="7" t="s">
         <v>42</v>
       </c>
@@ -2398,7 +2401,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A41" s="7" t="s">
         <v>42</v>
       </c>
@@ -2421,7 +2424,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A42" s="7" t="s">
         <v>42</v>
       </c>
@@ -2444,7 +2447,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A43" s="7" t="s">
         <v>42</v>
       </c>
@@ -2467,7 +2470,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A44" s="7" t="s">
         <v>42</v>
       </c>
@@ -2490,7 +2493,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A45" s="7" t="s">
         <v>42</v>
       </c>
@@ -2513,7 +2516,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A46" s="7" t="s">
         <v>42</v>
       </c>
@@ -2536,7 +2539,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A47" s="7" t="s">
         <v>42</v>
       </c>
@@ -2559,7 +2562,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A48" s="7" t="s">
         <v>42</v>
       </c>
@@ -2582,7 +2585,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A49" s="7" t="s">
         <v>42</v>
       </c>
@@ -2605,7 +2608,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A50" s="7" t="s">
         <v>42</v>
       </c>
@@ -2628,7 +2631,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A51" s="7" t="s">
         <v>42</v>
       </c>
@@ -2651,7 +2654,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A52" s="7" t="s">
         <v>42</v>
       </c>
@@ -2674,7 +2677,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A53" s="7" t="s">
         <v>42</v>
       </c>
@@ -2697,7 +2700,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A54" s="7" t="s">
         <v>42</v>
       </c>
@@ -2720,7 +2723,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A55" s="7" t="s">
         <v>42</v>
       </c>
@@ -2743,7 +2746,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A56" s="7" t="s">
         <v>42</v>
       </c>
@@ -2766,7 +2769,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A57" s="7" t="s">
         <v>42</v>
       </c>
@@ -2789,7 +2792,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A58" s="7" t="s">
         <v>42</v>
       </c>
@@ -2812,7 +2815,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A59" s="7" t="s">
         <v>42</v>
       </c>
@@ -2835,7 +2838,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A60" s="7" t="s">
         <v>42</v>
       </c>
@@ -2858,7 +2861,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A61" s="7" t="s">
         <v>42</v>
       </c>
@@ -2881,7 +2884,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A62" s="7" t="s">
         <v>42</v>
       </c>
@@ -2904,7 +2907,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A63" s="7" t="s">
         <v>42</v>
       </c>
@@ -2927,7 +2930,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A64" s="7" t="s">
         <v>42</v>
       </c>
@@ -2950,7 +2953,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A65" s="7" t="s">
         <v>42</v>
       </c>
@@ -2973,7 +2976,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A66" s="7" t="s">
         <v>42</v>
       </c>
@@ -2996,7 +2999,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A67" s="7" t="s">
         <v>42</v>
       </c>
@@ -3019,7 +3022,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A68" s="7" t="s">
         <v>42</v>
       </c>
@@ -3042,7 +3045,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A69" s="7" t="s">
         <v>42</v>
       </c>
@@ -3065,7 +3068,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A70" s="7" t="s">
         <v>42</v>
       </c>
@@ -3088,7 +3091,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A71" s="7" t="s">
         <v>42</v>
       </c>
@@ -3111,7 +3114,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A72" s="7" t="s">
         <v>42</v>
       </c>
@@ -3134,7 +3137,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A73" s="7" t="s">
         <v>42</v>
       </c>
@@ -3157,7 +3160,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A74" s="7" t="s">
         <v>42</v>
       </c>
@@ -3180,7 +3183,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A75" s="7" t="s">
         <v>42</v>
       </c>
@@ -3203,7 +3206,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A76" s="7" t="s">
         <v>42</v>
       </c>
@@ -3226,7 +3229,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A77" s="7" t="s">
         <v>42</v>
       </c>
@@ -3249,7 +3252,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A78" s="7" t="s">
         <v>42</v>
       </c>
@@ -3272,7 +3275,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A79" s="7" t="s">
         <v>42</v>
       </c>
@@ -3295,7 +3298,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A80" s="7" t="s">
         <v>42</v>
       </c>
@@ -3318,7 +3321,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A81" s="7" t="s">
         <v>42</v>
       </c>
@@ -3341,7 +3344,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A82" s="7" t="s">
         <v>42</v>
       </c>
@@ -3364,7 +3367,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A83" s="7" t="s">
         <v>42</v>
       </c>
@@ -3387,7 +3390,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A84" s="7" t="s">
         <v>42</v>
       </c>
@@ -3410,7 +3413,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A85" s="7" t="s">
         <v>42</v>
       </c>
@@ -3433,7 +3436,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A86" s="7" t="s">
         <v>42</v>
       </c>
@@ -3456,7 +3459,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A87" s="7" t="s">
         <v>42</v>
       </c>
@@ -3479,7 +3482,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A88" s="7" t="s">
         <v>42</v>
       </c>
@@ -3502,7 +3505,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A89" s="7" t="s">
         <v>42</v>
       </c>
@@ -3525,7 +3528,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A90" s="7" t="s">
         <v>42</v>
       </c>
@@ -3548,7 +3551,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A91" s="7" t="s">
         <v>42</v>
       </c>
@@ -3571,7 +3574,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A92" s="7" t="s">
         <v>42</v>
       </c>
@@ -3594,7 +3597,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A93" s="7" t="s">
         <v>42</v>
       </c>
@@ -3617,7 +3620,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A94" s="7" t="s">
         <v>42</v>
       </c>
@@ -3640,7 +3643,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A95" s="7" t="s">
         <v>42</v>
       </c>
@@ -3663,7 +3666,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A96" s="7" t="s">
         <v>42</v>
       </c>
@@ -3686,7 +3689,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A97" s="7" t="s">
         <v>42</v>
       </c>
@@ -3709,7 +3712,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A98" s="7" t="s">
         <v>42</v>
       </c>
@@ -3732,7 +3735,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A99" s="7" t="s">
         <v>42</v>
       </c>
@@ -3755,7 +3758,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A100" s="7" t="s">
         <v>42</v>
       </c>
@@ -3778,7 +3781,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A101" s="7" t="s">
         <v>42</v>
       </c>
@@ -3801,7 +3804,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A102" s="7" t="s">
         <v>42</v>
       </c>
@@ -3824,7 +3827,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A103" s="7" t="s">
         <v>42</v>
       </c>
@@ -3847,7 +3850,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A104" s="7" t="s">
         <v>42</v>
       </c>
@@ -3870,7 +3873,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A105" s="7" t="s">
         <v>42</v>
       </c>
@@ -3893,7 +3896,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A106" s="7" t="s">
         <v>42</v>
       </c>
@@ -3916,7 +3919,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A107" s="7" t="s">
         <v>42</v>
       </c>
@@ -3939,7 +3942,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A108" s="7" t="s">
         <v>42</v>
       </c>
@@ -3962,7 +3965,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="109" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A109" s="7" t="s">
         <v>42</v>
       </c>
@@ -3985,7 +3988,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A110" s="7" t="s">
         <v>42</v>
       </c>
@@ -4008,7 +4011,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="111" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A111" s="7" t="s">
         <v>42</v>
       </c>
@@ -4031,7 +4034,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="112" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A112" s="7" t="s">
         <v>42</v>
       </c>
@@ -4054,7 +4057,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="113" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A113" s="7" t="s">
         <v>42</v>
       </c>
@@ -4077,7 +4080,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="114" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A114" s="7" t="s">
         <v>42</v>
       </c>
@@ -4100,7 +4103,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="115" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A115" s="7" t="s">
         <v>42</v>
       </c>
@@ -4123,7 +4126,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="116" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A116" s="7" t="s">
         <v>42</v>
       </c>
@@ -4146,7 +4149,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="117" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A117" s="7" t="s">
         <v>42</v>
       </c>
@@ -4169,7 +4172,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="118" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A118" s="7" t="s">
         <v>42</v>
       </c>
@@ -4192,7 +4195,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="119" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A119" s="7" t="s">
         <v>42</v>
       </c>
@@ -4215,7 +4218,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="120" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A120" s="7" t="s">
         <v>42</v>
       </c>
@@ -4238,7 +4241,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="121" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A121" s="7" t="s">
         <v>42</v>
       </c>
@@ -4261,7 +4264,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="122" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A122" s="7" t="s">
         <v>42</v>
       </c>
@@ -4284,7 +4287,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="123" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A123" s="7" t="s">
         <v>42</v>
       </c>
@@ -4307,7 +4310,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="124" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A124" s="7" t="s">
         <v>42</v>
       </c>
@@ -4330,7 +4333,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="125" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A125" s="7" t="s">
         <v>42</v>
       </c>
@@ -4353,7 +4356,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="126" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A126" s="7" t="s">
         <v>42</v>
       </c>
@@ -4376,7 +4379,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="127" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A127" s="7" t="s">
         <v>42</v>
       </c>
@@ -4399,7 +4402,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="128" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A128" s="7" t="s">
         <v>42</v>
       </c>
@@ -4422,7 +4425,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="129" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A129" s="7" t="s">
         <v>42</v>
       </c>
@@ -4445,7 +4448,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="130" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A130" s="7" t="s">
         <v>42</v>
       </c>
@@ -4468,7 +4471,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="131" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A131" s="7" t="s">
         <v>42</v>
       </c>
@@ -4491,7 +4494,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="132" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A132" s="7" t="s">
         <v>42</v>
       </c>
@@ -4514,7 +4517,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="133" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A133" s="7" t="s">
         <v>42</v>
       </c>
@@ -4537,7 +4540,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="134" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A134" s="7" t="s">
         <v>42</v>
       </c>
@@ -4560,7 +4563,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="135" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A135" s="7" t="s">
         <v>42</v>
       </c>
@@ -4583,7 +4586,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="136" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A136" s="7" t="s">
         <v>42</v>
       </c>
@@ -4606,7 +4609,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="137" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A137" s="7" t="s">
         <v>42</v>
       </c>
@@ -4629,7 +4632,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="138" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A138" s="7" t="s">
         <v>42</v>
       </c>
@@ -4652,7 +4655,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="139" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A139" s="7" t="s">
         <v>42</v>
       </c>
@@ -4675,7 +4678,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="140" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A140" s="7" t="s">
         <v>42</v>
       </c>
@@ -4698,7 +4701,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="141" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A141" s="7" t="s">
         <v>42</v>
       </c>
@@ -4721,7 +4724,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="142" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A142" s="7" t="s">
         <v>42</v>
       </c>
@@ -4744,7 +4747,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="143" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A143" s="7" t="s">
         <v>42</v>
       </c>
@@ -4767,7 +4770,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="144" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A144" s="7" t="s">
         <v>42</v>
       </c>
@@ -4790,7 +4793,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="145" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A145" s="7" t="s">
         <v>42</v>
       </c>
@@ -4813,7 +4816,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="146" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A146" s="7" t="s">
         <v>42</v>
       </c>
@@ -4836,7 +4839,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="147" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A147" s="7" t="s">
         <v>42</v>
       </c>
@@ -4859,7 +4862,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="148" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A148" s="7" t="s">
         <v>42</v>
       </c>
@@ -4882,7 +4885,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="149" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A149" s="7" t="s">
         <v>42</v>
       </c>
@@ -4905,7 +4908,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="150" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A150" s="7" t="s">
         <v>42</v>
       </c>
@@ -4928,7 +4931,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="151" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A151" s="7" t="s">
         <v>42</v>
       </c>
@@ -4951,7 +4954,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="152" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A152" s="7" t="s">
         <v>42</v>
       </c>
@@ -4974,7 +4977,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="153" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A153" s="7" t="s">
         <v>42</v>
       </c>
@@ -4997,7 +5000,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="154" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A154" s="7" t="s">
         <v>42</v>
       </c>
@@ -5020,7 +5023,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="155" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A155" s="7" t="s">
         <v>42</v>
       </c>
@@ -5043,7 +5046,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="156" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A156" s="7" t="s">
         <v>42</v>
       </c>
@@ -5066,7 +5069,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="157" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A157" s="7" t="s">
         <v>42</v>
       </c>
@@ -5089,7 +5092,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="158" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A158" s="7" t="s">
         <v>42</v>
       </c>
@@ -5112,7 +5115,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="159" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A159" s="7" t="s">
         <v>42</v>
       </c>
@@ -5135,7 +5138,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="160" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A160" s="7" t="s">
         <v>42</v>
       </c>
@@ -5158,7 +5161,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="161" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A161" s="7" t="s">
         <v>42</v>
       </c>
@@ -5181,7 +5184,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="162" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A162" s="7" t="s">
         <v>42</v>
       </c>
@@ -5204,7 +5207,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="163" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A163" s="7" t="s">
         <v>42</v>
       </c>
@@ -5227,7 +5230,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="164" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A164" s="7" t="s">
         <v>42</v>
       </c>
@@ -5250,7 +5253,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="165" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A165" s="7" t="s">
         <v>42</v>
       </c>
@@ -5273,7 +5276,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="166" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A166" s="7" t="s">
         <v>42</v>
       </c>
@@ -5296,7 +5299,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="167" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A167" s="7" t="s">
         <v>42</v>
       </c>
@@ -5319,7 +5322,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="168" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A168" s="7" t="s">
         <v>42</v>
       </c>
@@ -5342,7 +5345,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="169" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A169" s="7" t="s">
         <v>42</v>
       </c>
@@ -5365,7 +5368,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="170" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A170" s="7" t="s">
         <v>42</v>
       </c>
@@ -5388,7 +5391,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="171" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A171" s="7" t="s">
         <v>42</v>
       </c>
@@ -5411,7 +5414,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="172" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A172" s="7" t="s">
         <v>42</v>
       </c>
@@ -5434,7 +5437,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="173" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A173" s="7" t="s">
         <v>42</v>
       </c>
@@ -5457,7 +5460,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="174" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A174" s="7" t="s">
         <v>42</v>
       </c>
@@ -5480,7 +5483,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="175" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A175" s="7" t="s">
         <v>42</v>
       </c>
@@ -5503,7 +5506,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="176" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A176" s="7" t="s">
         <v>42</v>
       </c>
@@ -5526,7 +5529,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="177" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A177" s="7" t="s">
         <v>42</v>
       </c>
@@ -5549,7 +5552,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="178" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A178" s="7" t="s">
         <v>42</v>
       </c>
@@ -5572,7 +5575,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="179" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A179" s="7" t="s">
         <v>42</v>
       </c>
@@ -5595,7 +5598,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="180" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A180" s="7" t="s">
         <v>42</v>
       </c>
@@ -5618,7 +5621,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="181" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A181" s="7" t="s">
         <v>42</v>
       </c>
@@ -5641,7 +5644,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="182" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A182" s="7" t="s">
         <v>42</v>
       </c>
@@ -5664,7 +5667,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="183" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A183" s="7" t="s">
         <v>42</v>
       </c>
@@ -5687,7 +5690,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="184" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A184" s="7" t="s">
         <v>42</v>
       </c>
@@ -5710,7 +5713,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="185" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A185" s="7" t="s">
         <v>42</v>
       </c>
@@ -5733,7 +5736,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="186" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A186" s="7" t="s">
         <v>42</v>
       </c>
@@ -5756,7 +5759,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="187" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A187" s="7" t="s">
         <v>42</v>
       </c>
@@ -5779,7 +5782,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="188" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A188" s="7" t="s">
         <v>42</v>
       </c>
@@ -5802,7 +5805,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="189" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A189" s="7" t="s">
         <v>42</v>
       </c>
@@ -5825,7 +5828,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="190" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A190" s="7" t="s">
         <v>42</v>
       </c>
@@ -5848,7 +5851,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="191" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A191" s="7" t="s">
         <v>42</v>
       </c>
@@ -5871,7 +5874,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="192" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A192" s="7" t="s">
         <v>42</v>
       </c>
@@ -5894,7 +5897,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="193" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A193" s="7" t="s">
         <v>42</v>
       </c>
@@ -5917,7 +5920,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="194" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A194" s="7" t="s">
         <v>42</v>
       </c>
@@ -5940,7 +5943,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="195" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A195" s="7" t="s">
         <v>42</v>
       </c>
@@ -5963,7 +5966,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="196" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A196" s="7" t="s">
         <v>42</v>
       </c>
@@ -5986,7 +5989,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="197" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A197" s="7" t="s">
         <v>42</v>
       </c>
@@ -6009,7 +6012,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="198" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A198" s="7" t="s">
         <v>42</v>
       </c>
@@ -6032,7 +6035,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="199" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A199" s="7" t="s">
         <v>42</v>
       </c>
@@ -6055,7 +6058,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="200" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A200" s="7" t="s">
         <v>42</v>
       </c>
@@ -6078,7 +6081,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="201" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A201" s="7" t="s">
         <v>42</v>
       </c>
@@ -6101,7 +6104,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="202" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A202" s="7" t="s">
         <v>42</v>
       </c>
@@ -6124,7 +6127,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="203" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A203" s="7" t="s">
         <v>42</v>
       </c>
@@ -6147,7 +6150,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="204" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A204" s="7" t="s">
         <v>42</v>
       </c>
@@ -6170,7 +6173,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="205" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A205" s="7" t="s">
         <v>42</v>
       </c>
@@ -6193,7 +6196,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="206" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A206" s="7" t="s">
         <v>42</v>
       </c>
@@ -6216,7 +6219,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="207" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A207" s="7" t="s">
         <v>42</v>
       </c>
@@ -6239,7 +6242,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="208" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A208" s="7" t="s">
         <v>42</v>
       </c>
@@ -6262,7 +6265,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="209" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A209" s="7" t="s">
         <v>42</v>
       </c>
@@ -6285,7 +6288,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="210" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A210" s="7" t="s">
         <v>42</v>
       </c>
@@ -6308,7 +6311,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="211" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A211" s="7" t="s">
         <v>42</v>
       </c>
@@ -6331,7 +6334,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="212" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A212" s="7" t="s">
         <v>42</v>
       </c>
@@ -6354,7 +6357,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="213" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A213" s="7" t="s">
         <v>42</v>
       </c>
@@ -6377,7 +6380,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="214" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A214" s="7" t="s">
         <v>42</v>
       </c>
@@ -6400,7 +6403,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="215" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A215" s="7" t="s">
         <v>42</v>
       </c>
@@ -6423,7 +6426,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="216" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A216" s="7" t="s">
         <v>42</v>
       </c>
@@ -6446,7 +6449,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="217" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A217" s="7" t="s">
         <v>42</v>
       </c>
@@ -6469,7 +6472,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="218" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A218" s="7" t="s">
         <v>42</v>
       </c>
@@ -6492,7 +6495,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="219" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A219" s="7" t="s">
         <v>42</v>
       </c>
@@ -6515,7 +6518,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="220" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A220" s="7" t="s">
         <v>42</v>
       </c>
@@ -6538,7 +6541,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="221" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A221" s="7" t="s">
         <v>42</v>
       </c>
@@ -6561,7 +6564,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="222" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A222" s="7" t="s">
         <v>42</v>
       </c>
@@ -6584,7 +6587,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="223" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A223" s="7" t="s">
         <v>42</v>
       </c>
@@ -6607,7 +6610,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="224" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A224" s="7" t="s">
         <v>42</v>
       </c>
@@ -6630,7 +6633,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="225" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A225" s="7" t="s">
         <v>42</v>
       </c>
@@ -6653,7 +6656,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="226" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A226" s="7" t="s">
         <v>42</v>
       </c>
@@ -6676,7 +6679,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="227" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A227" s="7" t="s">
         <v>42</v>
       </c>
@@ -6699,7 +6702,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="228" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A228" s="7" t="s">
         <v>42</v>
       </c>
@@ -6722,7 +6725,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="229" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A229" s="7" t="s">
         <v>42</v>
       </c>
@@ -6745,7 +6748,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="230" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A230" s="7" t="s">
         <v>42</v>
       </c>
@@ -6768,7 +6771,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="231" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A231" s="7" t="s">
         <v>42</v>
       </c>
@@ -6791,7 +6794,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="232" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A232" s="7" t="s">
         <v>42</v>
       </c>
@@ -6814,7 +6817,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="233" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A233" s="7" t="s">
         <v>42</v>
       </c>
@@ -6837,7 +6840,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="234" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A234" s="7" t="s">
         <v>42</v>
       </c>
@@ -6860,7 +6863,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="235" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A235" s="7" t="s">
         <v>42</v>
       </c>
@@ -6883,7 +6886,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="236" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A236" s="7" t="s">
         <v>42</v>
       </c>
@@ -6906,7 +6909,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="237" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A237" s="7" t="s">
         <v>42</v>
       </c>
@@ -6929,7 +6932,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="238" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A238" s="7" t="s">
         <v>42</v>
       </c>
@@ -6952,7 +6955,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="239" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A239" s="7" t="s">
         <v>42</v>
       </c>
@@ -6975,7 +6978,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="240" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A240" s="7" t="s">
         <v>42</v>
       </c>
@@ -6998,7 +7001,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="241" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A241" s="7" t="s">
         <v>42</v>
       </c>
@@ -7021,7 +7024,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="242" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="242" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A242" s="7" t="s">
         <v>42</v>
       </c>
@@ -7044,7 +7047,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="243" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="243" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A243" s="7" t="s">
         <v>42</v>
       </c>
@@ -7067,7 +7070,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="244" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A244" s="7" t="s">
         <v>42</v>
       </c>
@@ -7090,7 +7093,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="245" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="245" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A245" s="7" t="s">
         <v>42</v>
       </c>
@@ -7113,7 +7116,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="246" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="246" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A246" s="7" t="s">
         <v>42</v>
       </c>
@@ -7136,7 +7139,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="247" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="247" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A247" s="7" t="s">
         <v>42</v>
       </c>
@@ -7159,7 +7162,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="248" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="248" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A248" s="7" t="s">
         <v>42</v>
       </c>
@@ -7182,7 +7185,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="249" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A249" s="7" t="s">
         <v>42</v>
       </c>
@@ -7205,7 +7208,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="250" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="250" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A250" s="9" t="s">
         <v>42</v>
       </c>
@@ -7229,21 +7232,13 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:G250" xr:uid="{156349CF-6280-4CD0-803A-013CF8C0A2F2}"/>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100DC8BB5B596CFDD4794B3344F0E8F53A4" ma:contentTypeVersion="15" ma:contentTypeDescription="Criar um novo documento." ma:contentTypeScope="" ma:versionID="9a7078cd21229583650f2264465a1c40">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="20d57abc-823c-4051-a81a-1a0a01a8f39e" xmlns:ns3="54c5ab46-7543-4aba-b0fa-79d6a199bef5" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4e45437c47114f519c494620e3e4bb67" ns2:_="" ns3:_="">
     <xsd:import namespace="20d57abc-823c-4051-a81a-1a0a01a8f39e"/>
@@ -7478,6 +7473,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -7490,14 +7494,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{39FDDE8C-0A1E-4704-A23F-A36DCD77389B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3A89C6CB-9C03-4AE9-BB36-D0188DD65F32}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -7516,6 +7512,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{39FDDE8C-0A1E-4704-A23F-A36DCD77389B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8C58ACE5-5395-40A6-B201-757ED1E50D7A}">
   <ds:schemaRefs>

</xml_diff>